<commit_message>
Update workspace at /fa
</commit_message>
<xml_diff>
--- a/public/fa/example-project.xlsx
+++ b/public/fa/example-project.xlsx
@@ -418,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -576,9 +576,17 @@
         <v>Cards, Disputes, Automation</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Stack</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Java, Spring Boot, PostgreSQL, Swagger, Postman, Docker</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>